<commit_message>
Screen SPOT/PFE/UPS from Darryl list to close out the day
SPOT cleared to Ready for Tier 1 (~3.67 quant-only; sole weak spot was
relative_strength, but the Fidelity scan reinforced rather than
undercut the read this time -- Bullish 7.2/10 consensus, zero Sell
ratings, Evercore raised its target to $700 on 9/29). PFE and UPS both
rejected as decisive floor failures (~2.56 and ~2.44), each with two
indicators at the literal floor -- same territory as GXO's earlier
rejection. Journal row 70; CANDIDATES LIST.xlsx Screen_Candidates
updated for all three. 17 Darryl names remain unscreened, plus UNH/ACN
still at Watch status from earlier today.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CANDIDATES LIST.xlsx
+++ b/CANDIDATES LIST.xlsx
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="611" uniqueCount="265">
   <si>
     <t xml:space="preserve">Ticker</t>
   </si>
@@ -178,6 +178,12 @@
     <t xml:space="preserve">Darryl</t>
   </si>
   <si>
+    <t xml:space="preserve">Ready for Tier 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initial quant Tier 1 screen 9/30/26: ~3.67 quant-only (strong -- fcf_yield 4, rev growth 4, fcf margin 4 expanding, valuation 4 discount, analyst consensus 5, technical 4, ROIC 5 [44.6% vs WACC 11.1%, +33.5pp spread]; only weak spot relative_strength=1, blended -29.7% vs SPY). Same fundamentals-strong-but-price-lagging pattern as ACN -- ran the Fidelity scan on it specifically. Unlike ACN/ADBE/UNH, this one reinforced rather than undercut the quant read: Equity Summary Score Bullish (7.2/10), zero Sell ratings across 6 firms, Evercore ISI raised its price target to $700 on 9/29, short interest declining (6.12M -&gt; 4.52M). Price weakness reads as giving back part of a large 2yr (+32%) / 5yr (+121%) run after a Q2 EPS miss, not a structural deterioration -- meaningfully different pattern from ADBE's multi-year decline. Cleared to Ready for Tier 1; full Tier 1-3 scoring not done yet (separate pass, like ABT/SLB). Reports Q3 earnings 10/22/26. See Journal row 70.</t>
+  </si>
+  <si>
     <t xml:space="preserve">KGS</t>
   </si>
   <si>
@@ -190,9 +196,6 @@
     <t xml:space="preserve">Oil &amp; Gas Equipment &amp; Services</t>
   </si>
   <si>
-    <t xml:space="preserve">Ready for Tier 1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fresh Tier 1 quant screen 9/11/26: FCF Yield=4, Rev Growth=4, FCF Margin=4 (Tier1 Wtd Avg=4.0 on known indicators). Moat/Rev Visibility not yet assessed (Part 12, qualitative). Added to Scoring (row 48) and Monitor &amp; Recheck Triggers as Watch List.</t>
   </si>
   <si>
@@ -322,6 +325,9 @@
     <t xml:space="preserve">Pfizer Inc.</t>
   </si>
   <si>
+    <t xml:space="preserve">Initial quant Tier 1 screen 9/30/26: ~2.56 quant-only, decisive floor failure -- two indicators at the literal floor: revenue_growth_consistency=1 (negative CAGR -14.8%) and roic_vs_wacc=1 (ROIC 5.1% vs WACC 6.2%, actually value-destroying, spread -1.1pp). Same territory as GXO's rejection. Analyst consensus also weak (36% buy-equivalent, 7% negative). Rejected -- fundamental, not a data-quality artifact. See Journal row 70.</t>
+  </si>
+  <si>
     <t xml:space="preserve">UNH</t>
   </si>
   <si>
@@ -449,6 +455,9 @@
   </si>
   <si>
     <t xml:space="preserve">United Parcel Service, Inc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Initial quant Tier 1 screen 9/30/26: ~2.44 quant-only, decisive floor failure -- two indicators at the literal floor: revenue_growth_consistency=1 (negative CAGR -4.0%) and technical_trend=1 (200w MA below, MACD not ok, Supertrend bearish -- broadly negative across the board). Same territory as GXO's rejection. Rejected -- fundamental, not a data-quality artifact. See Journal row 70.</t>
   </si>
   <si>
     <t xml:space="preserve">CCI</t>
@@ -2060,12 +2069,14 @@
       </c>
       <c r="H4" s="5"/>
       <c r="I4" s="5" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="J4" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="K4" s="9"/>
+      <c r="K4" s="9" t="s">
+        <v>30</v>
+      </c>
       <c r="N4" s="11" t="s">
         <v>22</v>
       </c>
@@ -2075,16 +2086,16 @@
     </row>
     <row r="5" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C5,$N$3:$N$13,0)),0.25)</f>
@@ -2098,16 +2109,16 @@
       </c>
       <c r="H5" s="5"/>
       <c r="I5" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J5" s="8" t="n">
         <v>46264</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O5" s="12" t="n">
         <v>0</v>
@@ -2115,16 +2126,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C6,$N$3:$N$13,0)),0.25)</f>
@@ -2145,7 +2156,7 @@
       </c>
       <c r="K6" s="9"/>
       <c r="N6" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O6" s="12" t="n">
         <v>0</v>
@@ -2153,16 +2164,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C7,$N$3:$N$13,0)),0.25)</f>
@@ -2176,16 +2187,16 @@
       </c>
       <c r="H7" s="5"/>
       <c r="I7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J7" s="8" t="n">
+        <v>46244</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="N7" s="11" t="s">
         <v>33</v>
-      </c>
-      <c r="J7" s="8" t="n">
-        <v>46244</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="N7" s="11" t="s">
-        <v>31</v>
       </c>
       <c r="O7" s="12" t="n">
         <v>0</v>
@@ -2193,16 +2204,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C8,$N$3:$N$13,0)),0.25)</f>
@@ -2216,16 +2227,16 @@
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J8" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="O8" s="12" t="n">
         <v>0</v>
@@ -2233,16 +2244,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E9" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C9,$N$3:$N$13,0)),0.25)</f>
@@ -2256,16 +2267,16 @@
       </c>
       <c r="H9" s="5"/>
       <c r="I9" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N9" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O9" s="12" t="n">
         <v>0.0342</v>
@@ -2273,16 +2284,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E10" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C10,$N$3:$N$13,0)),0.25)</f>
@@ -2303,7 +2314,7 @@
       </c>
       <c r="K10" s="9"/>
       <c r="N10" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O10" s="12" t="n">
         <v>0.0119</v>
@@ -2311,16 +2322,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E11" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C11,$N$3:$N$13,0)),0.25)</f>
@@ -2341,7 +2352,7 @@
       </c>
       <c r="K11" s="9"/>
       <c r="N11" s="11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="O11" s="12" t="n">
         <v>0.0249</v>
@@ -2349,16 +2360,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E12" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C12,$N$3:$N$13,0)),0.25)</f>
@@ -2379,7 +2390,7 @@
       </c>
       <c r="K12" s="9"/>
       <c r="N12" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O12" s="12" t="n">
         <v>0.2586</v>
@@ -2387,16 +2398,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E13" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C13,$N$3:$N$13,0)),0.25)</f>
@@ -2417,7 +2428,7 @@
       </c>
       <c r="K13" s="9"/>
       <c r="N13" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O13" s="12" t="n">
         <v>0</v>
@@ -2425,16 +2436,16 @@
     </row>
     <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E14" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C14,$N$3:$N$13,0)),0.25)</f>
@@ -2454,21 +2465,21 @@
         <v>46264</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E15" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C15,$N$3:$N$13,0)),0.25)</f>
@@ -2491,16 +2502,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E16" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C16,$N$3:$N$13,0)),0.25)</f>
@@ -2514,25 +2525,27 @@
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="J16" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="K16" s="9"/>
+      <c r="K16" s="9" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E17" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C17,$N$3:$N$13,0)),0.25)</f>
@@ -2546,27 +2559,27 @@
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="J17" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E18" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C18,$N$3:$N$13,0)),0.25)</f>
@@ -2589,16 +2602,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E19" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C19,$N$3:$N$13,0)),0.25)</f>
@@ -2612,27 +2625,27 @@
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J19" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E20" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C20,$N$3:$N$13,0)),0.25)</f>
@@ -2655,16 +2668,16 @@
     </row>
     <row r="21" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C21,$N$3:$N$13,0)),0.25)</f>
@@ -2684,21 +2697,21 @@
         <v>46264</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E22" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C22,$N$3:$N$13,0)),0.25)</f>
@@ -2712,27 +2725,27 @@
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J22" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E23" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C23,$N$3:$N$13,0)),0.25)</f>
@@ -2752,21 +2765,21 @@
         <v>46264</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E24" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C24,$N$3:$N$13,0)),0.25)</f>
@@ -2786,21 +2799,21 @@
         <v>46244</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E25" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C25,$N$3:$N$13,0)),0.25)</f>
@@ -2820,21 +2833,21 @@
         <v>46244</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E26" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C26,$N$3:$N$13,0)),0.25)</f>
@@ -2854,21 +2867,21 @@
         <v>46244</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E27" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C27,$N$3:$N$13,0)),0.25)</f>
@@ -2891,16 +2904,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E28" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C28,$N$3:$N$13,0)),0.25)</f>
@@ -2923,16 +2936,16 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E29" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C29,$N$3:$N$13,0)),0.25)</f>
@@ -2946,25 +2959,27 @@
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="5" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="J29" s="8" t="n">
         <v>46244</v>
       </c>
-      <c r="K29" s="9"/>
+      <c r="K29" s="9" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="E30" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C30,$N$3:$N$13,0)),0.25)</f>
@@ -2978,27 +2993,27 @@
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J30" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E31" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C31,$N$3:$N$13,0)),0.25)</f>
@@ -3018,21 +3033,21 @@
         <v>46244</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E32" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C32,$N$3:$N$13,0)),0.25)</f>
@@ -3046,27 +3061,27 @@
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="J32" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E33" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C33,$N$3:$N$13,0)),0.25)</f>
@@ -3086,21 +3101,21 @@
         <v>46264</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="95.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E34" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C34,$N$3:$N$13,0)),0.25)</f>
@@ -3120,21 +3135,21 @@
         <v>46264</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E35" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C35,$N$3:$N$13,0)),0.25)</f>
@@ -3154,21 +3169,21 @@
         <v>46244</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="E36" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C36,$N$3:$N$13,0)),0.25)</f>
@@ -3188,21 +3203,21 @@
         <v>46264</v>
       </c>
       <c r="K36" s="9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E37" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C37,$N$3:$N$13,0)),0.25)</f>
@@ -3225,16 +3240,16 @@
     </row>
     <row r="38" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="E38" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C38,$N$3:$N$13,0)),0.25)</f>
@@ -3254,21 +3269,21 @@
         <v>46264</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E39" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C39,$N$3:$N$13,0)),0.25)</f>
@@ -3291,16 +3306,16 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E40" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C40,$N$3:$N$13,0)),0.25)</f>
@@ -3313,10 +3328,10 @@
         <v>28</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J40" s="8" t="n">
         <v>46244</v>
@@ -3325,16 +3340,16 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E41" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C41,$N$3:$N$13,0)),0.25)</f>
@@ -3347,10 +3362,10 @@
         <v>28</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J41" s="8" t="n">
         <v>46244</v>
@@ -3359,16 +3374,16 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E42" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C42,$N$3:$N$13,0)),0.25)</f>
@@ -3381,10 +3396,10 @@
         <v>28</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J42" s="8" t="n">
         <v>46244</v>
@@ -3393,16 +3408,16 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E43" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C43,$N$3:$N$13,0)),0.25)</f>
@@ -3415,10 +3430,10 @@
         <v>28</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J43" s="8" t="n">
         <v>46244</v>
@@ -3427,16 +3442,16 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E44" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C44,$N$3:$N$13,0)),0.25)</f>
@@ -3449,10 +3464,10 @@
         <v>28</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J44" s="8" t="n">
         <v>46244</v>
@@ -3461,16 +3476,16 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E45" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C45,$N$3:$N$13,0)),0.25)</f>
@@ -3483,10 +3498,10 @@
         <v>28</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J45" s="8" t="n">
         <v>46244</v>
@@ -3495,16 +3510,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E46" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C46,$N$3:$N$13,0)),0.25)</f>
@@ -3517,10 +3532,10 @@
         <v>28</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I46" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J46" s="8" t="n">
         <v>46244</v>
@@ -3529,16 +3544,16 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E47" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C47,$N$3:$N$13,0)),0.25)</f>
@@ -3551,10 +3566,10 @@
         <v>28</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J47" s="8" t="n">
         <v>46244</v>
@@ -3563,16 +3578,16 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E48" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C48,$N$3:$N$13,0)),0.25)</f>
@@ -3585,10 +3600,10 @@
         <v>28</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J48" s="8" t="n">
         <v>46244</v>
@@ -3597,16 +3612,16 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E49" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C49,$N$3:$N$13,0)),0.25)</f>
@@ -3619,10 +3634,10 @@
         <v>28</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>46244</v>
@@ -3631,16 +3646,16 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E50" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C50,$N$3:$N$13,0)),0.25)</f>
@@ -3653,10 +3668,10 @@
         <v>28</v>
       </c>
       <c r="H50" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="J50" s="8" t="n">
         <v>46244</v>
@@ -3665,16 +3680,16 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>14</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E51" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C51,$N$3:$N$13,0)),0.25)</f>
@@ -3687,10 +3702,10 @@
         <v>28</v>
       </c>
       <c r="H51" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I51" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J51" s="8" t="n">
         <v>46244</v>
@@ -3699,16 +3714,16 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>14</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E52" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C52,$N$3:$N$13,0)),0.25)</f>
@@ -3721,10 +3736,10 @@
         <v>28</v>
       </c>
       <c r="H52" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I52" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J52" s="8" t="n">
         <v>46244</v>
@@ -3733,16 +3748,16 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>22</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="E53" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C53,$N$3:$N$13,0)),0.25)</f>
@@ -3755,10 +3770,10 @@
         <v>28</v>
       </c>
       <c r="H53" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I53" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J53" s="8" t="n">
         <v>46244</v>
@@ -3767,16 +3782,16 @@
     </row>
     <row r="54" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D54" s="5" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="E54" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C54,$N$3:$N$13,0)),0.25)</f>
@@ -3789,30 +3804,30 @@
         <v>28</v>
       </c>
       <c r="H54" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I54" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J54" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K54" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E55" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C55,$N$3:$N$13,0)),0.25)</f>
@@ -3825,30 +3840,30 @@
         <v>28</v>
       </c>
       <c r="H55" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I55" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J55" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K55" s="9" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D56" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E56" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C56,$N$3:$N$13,0)),0.25)</f>
@@ -3861,10 +3876,10 @@
         <v>28</v>
       </c>
       <c r="H56" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I56" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J56" s="8" t="n">
         <v>46244</v>
@@ -3873,16 +3888,16 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E57" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C57,$N$3:$N$13,0)),0.25)</f>
@@ -3895,10 +3910,10 @@
         <v>28</v>
       </c>
       <c r="H57" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I57" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J57" s="8" t="n">
         <v>46244</v>
@@ -3907,16 +3922,16 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="E58" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C58,$N$3:$N$13,0)),0.25)</f>
@@ -3929,10 +3944,10 @@
         <v>28</v>
       </c>
       <c r="H58" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I58" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J58" s="8" t="n">
         <v>46244</v>
@@ -3941,16 +3956,16 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E59" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C59,$N$3:$N$13,0)),0.25)</f>
@@ -3963,30 +3978,30 @@
         <v>28</v>
       </c>
       <c r="H59" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I59" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J59" s="8" t="n">
         <v>46244</v>
       </c>
       <c r="K59" s="9" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E60" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C60,$N$3:$N$13,0)),0.25)</f>
@@ -3999,10 +4014,10 @@
         <v>28</v>
       </c>
       <c r="H60" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I60" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J60" s="8" t="n">
         <v>46244</v>
@@ -4011,16 +4026,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E61" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C61,$N$3:$N$13,0)),0.25)</f>
@@ -4033,10 +4048,10 @@
         <v>28</v>
       </c>
       <c r="H61" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I61" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J61" s="8" t="n">
         <v>46244</v>
@@ -4045,16 +4060,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="E62" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C62,$N$3:$N$13,0)),0.25)</f>
@@ -4067,10 +4082,10 @@
         <v>28</v>
       </c>
       <c r="H62" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I62" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J62" s="8" t="n">
         <v>46244</v>
@@ -4079,16 +4094,16 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="E63" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C63,$N$3:$N$13,0)),0.25)</f>
@@ -4101,10 +4116,10 @@
         <v>28</v>
       </c>
       <c r="H63" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I63" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J63" s="8" t="n">
         <v>46244</v>
@@ -4113,16 +4128,16 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E64" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C64,$N$3:$N$13,0)),0.25)</f>
@@ -4135,10 +4150,10 @@
         <v>28</v>
       </c>
       <c r="H64" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I64" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J64" s="8" t="n">
         <v>46244</v>
@@ -4147,16 +4162,16 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E65" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C65,$N$3:$N$13,0)),0.25)</f>
@@ -4169,10 +4184,10 @@
         <v>28</v>
       </c>
       <c r="H65" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I65" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J65" s="8" t="n">
         <v>46244</v>
@@ -4181,16 +4196,16 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E66" s="6" t="n">
         <f aca="false">IFERROR(0.25-INDEX($O$3:$O$13,MATCH(C66,$N$3:$N$13,0)),0.25)</f>
@@ -4203,10 +4218,10 @@
         <v>28</v>
       </c>
       <c r="H66" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I66" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J66" s="8" t="n">
         <v>46244</v>
@@ -4306,79 +4321,79 @@
         <v>14</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>22</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H1" s="19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="I1" s="16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="J1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="K1" s="18" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L1" s="19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="M1" s="16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="N1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="O1" s="18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="P1" s="19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="Q1" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="R1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="S1" s="18" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="T1" s="19" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="U1" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="V1" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="W1" s="20" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="Z1" s="22" t="s">
         <v>2</v>
       </c>
       <c r="AA1" s="22" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="AB1" s="22" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" s="21" customFormat="true" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4419,63 +4434,63 @@
         <v>3</v>
       </c>
       <c r="AB2" s="25" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" s="21" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="27" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C3" s="29" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="D3" s="30" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E3" s="31"/>
       <c r="F3" s="32" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="G3" s="29" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H3" s="30" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I3" s="27" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="J3" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K3" s="29" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="L3" s="30"/>
       <c r="M3" s="27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="N3" s="28"/>
       <c r="O3" s="29" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="P3" s="30"/>
       <c r="Q3" s="27" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="R3" s="28"/>
       <c r="S3" s="29" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="T3" s="30"/>
       <c r="U3" s="27" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="V3" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="W3" s="33"/>
       <c r="Z3" s="25" t="s">
@@ -4485,133 +4500,133 @@
         <v>2</v>
       </c>
       <c r="AB3" s="25" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B4" s="35" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C4" s="36" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D4" s="37" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="E4" s="38" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F4" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G4" s="36" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="H4" s="30" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I4" s="38" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="J4" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="K4" s="38" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="L4" s="40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="M4" s="34" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="N4" s="35"/>
       <c r="O4" s="36" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="P4" s="37"/>
       <c r="Q4" s="34" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="R4" s="35"/>
       <c r="S4" s="36" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="T4" s="37"/>
       <c r="U4" s="38" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="V4" s="40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="Z4" s="25" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="AA4" s="26" t="n">
         <v>10</v>
       </c>
       <c r="AB4" s="25" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C5" s="36" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="37"/>
       <c r="E5" s="38" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F5" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="H5" s="30" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="I5" s="34" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="J5" s="35" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K5" s="36"/>
       <c r="L5" s="37"/>
       <c r="M5" s="34" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N5" s="35"/>
       <c r="O5" s="36" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P5" s="37"/>
       <c r="Q5" s="34"/>
       <c r="R5" s="35"/>
       <c r="S5" s="36" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="T5" s="37"/>
       <c r="U5" s="34"/>
       <c r="V5" s="35"/>
       <c r="Z5" s="25" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="AA5" s="26" t="n">
         <v>4</v>
       </c>
       <c r="AB5" s="25" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4620,51 +4635,51 @@
       <c r="C6" s="36"/>
       <c r="D6" s="37"/>
       <c r="E6" s="34" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F6" s="35" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H6" s="40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I6" s="34" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="J6" s="35" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="K6" s="36"/>
       <c r="L6" s="37"/>
       <c r="M6" s="34" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N6" s="35"/>
       <c r="O6" s="36" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="P6" s="37"/>
       <c r="Q6" s="34"/>
       <c r="R6" s="35"/>
       <c r="S6" s="38" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="T6" s="40" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="U6" s="34"/>
       <c r="V6" s="35"/>
       <c r="Z6" s="25" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="AA6" s="26" t="n">
         <v>6</v>
       </c>
       <c r="AB6" s="25" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4673,43 +4688,43 @@
       <c r="C7" s="36"/>
       <c r="D7" s="37"/>
       <c r="E7" s="41" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="F7" s="42" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G7" s="36"/>
       <c r="H7" s="37"/>
       <c r="I7" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J7" s="35"/>
       <c r="K7" s="36"/>
       <c r="L7" s="37"/>
       <c r="M7" s="34" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N7" s="35"/>
       <c r="O7" s="36" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="P7" s="37"/>
       <c r="Q7" s="34"/>
       <c r="R7" s="35"/>
       <c r="S7" s="36" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="34"/>
       <c r="V7" s="35"/>
       <c r="Z7" s="25" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AA7" s="26" t="n">
         <v>2</v>
       </c>
       <c r="AB7" s="25" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4719,22 +4734,22 @@
       <c r="D8" s="37"/>
       <c r="E8" s="43"/>
       <c r="F8" s="44" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="G8" s="36"/>
       <c r="H8" s="37"/>
       <c r="I8" s="34" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J8" s="35"/>
       <c r="K8" s="36"/>
       <c r="L8" s="37"/>
       <c r="M8" s="34" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N8" s="35"/>
       <c r="O8" s="36" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="P8" s="37"/>
       <c r="Q8" s="34"/>
@@ -4744,13 +4759,13 @@
       <c r="U8" s="34"/>
       <c r="V8" s="35"/>
       <c r="Z8" s="25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AA8" s="26" t="n">
         <v>9</v>
       </c>
       <c r="AB8" s="25" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4759,10 +4774,10 @@
       <c r="C9" s="36"/>
       <c r="D9" s="37"/>
       <c r="E9" s="45" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F9" s="46" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G9" s="36"/>
       <c r="H9" s="37"/>
@@ -4771,11 +4786,11 @@
       <c r="K9" s="36"/>
       <c r="L9" s="37"/>
       <c r="M9" s="34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N9" s="35"/>
       <c r="O9" s="36" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="P9" s="37"/>
       <c r="Q9" s="34"/>
@@ -4785,13 +4800,13 @@
       <c r="U9" s="34"/>
       <c r="V9" s="35"/>
       <c r="Z9" s="25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AA9" s="26" t="n">
         <v>8</v>
       </c>
       <c r="AB9" s="25" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4800,10 +4815,10 @@
       <c r="C10" s="36"/>
       <c r="D10" s="37"/>
       <c r="E10" s="34" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="F10" s="46" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G10" s="36"/>
       <c r="H10" s="37"/>
@@ -4812,11 +4827,11 @@
       <c r="K10" s="36"/>
       <c r="L10" s="37"/>
       <c r="M10" s="34" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N10" s="35"/>
       <c r="O10" s="36" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="P10" s="37"/>
       <c r="Q10" s="34"/>
@@ -4826,13 +4841,13 @@
       <c r="U10" s="34"/>
       <c r="V10" s="35"/>
       <c r="Z10" s="25" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AA10" s="26" t="n">
         <v>2</v>
       </c>
       <c r="AB10" s="25" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4841,10 +4856,10 @@
       <c r="C11" s="36"/>
       <c r="D11" s="37"/>
       <c r="E11" s="34" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="F11" s="46" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G11" s="36"/>
       <c r="H11" s="37"/>
@@ -4853,7 +4868,7 @@
       <c r="K11" s="36"/>
       <c r="L11" s="37"/>
       <c r="M11" s="34" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N11" s="35"/>
       <c r="O11" s="36"/>
@@ -4865,13 +4880,13 @@
       <c r="U11" s="34"/>
       <c r="V11" s="35"/>
       <c r="Z11" s="25" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AA11" s="26" t="n">
         <v>5</v>
       </c>
       <c r="AB11" s="25" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4881,7 +4896,7 @@
       <c r="D12" s="37"/>
       <c r="E12" s="43"/>
       <c r="F12" s="47" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G12" s="36"/>
       <c r="H12" s="37"/>
@@ -4890,7 +4905,7 @@
       <c r="K12" s="36"/>
       <c r="L12" s="37"/>
       <c r="M12" s="34" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="N12" s="35"/>
       <c r="O12" s="36"/>
@@ -4902,13 +4917,13 @@
       <c r="U12" s="34"/>
       <c r="V12" s="35"/>
       <c r="Z12" s="25" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="AA12" s="26" t="n">
         <v>2</v>
       </c>
       <c r="AB12" s="25" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4917,10 +4932,10 @@
       <c r="C13" s="36"/>
       <c r="D13" s="37"/>
       <c r="E13" s="45" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F13" s="46" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G13" s="36"/>
       <c r="H13" s="37"/>
@@ -4939,13 +4954,13 @@
       <c r="U13" s="34"/>
       <c r="V13" s="35"/>
       <c r="Z13" s="48" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="AA13" s="49" t="n">
         <v>1</v>
       </c>
       <c r="AB13" s="48" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4954,10 +4969,10 @@
       <c r="C14" s="36"/>
       <c r="D14" s="37"/>
       <c r="E14" s="34" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F14" s="35" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="G14" s="36"/>
       <c r="H14" s="37"/>
@@ -4982,10 +4997,10 @@
       <c r="C15" s="52"/>
       <c r="D15" s="53"/>
       <c r="E15" s="54" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F15" s="55" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G15" s="52"/>
       <c r="H15" s="53"/>
@@ -5163,15 +5178,15 @@
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E19" s="59" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E20" s="13" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="V20" s="60" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="W20" s="61" t="n">
         <f aca="false">COUNTIF($A$1:$V$15,"PASS")</f>
@@ -5184,7 +5199,7 @@
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="V21" s="60" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="W21" s="63" t="n">
         <f aca="false">COUNTIF($A$1:$V$15,"Avoid")</f>
@@ -5197,7 +5212,7 @@
     </row>
     <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="V22" s="60" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="W22" s="65" t="n">
         <f aca="false">SUM(W20:W21)</f>

</xml_diff>